<commit_message>
Update SS_mapping.xlsx via Streamlit
</commit_message>
<xml_diff>
--- a/SS_mapping.xlsx
+++ b/SS_mapping.xlsx
@@ -762,7 +762,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -820,7 +820,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -928,7 +928,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>

</xml_diff>